<commit_message>
Update reconciliation and normalization logic
</commit_message>
<xml_diff>
--- a/dummy.xlsx
+++ b/dummy.xlsx
@@ -29,8 +29,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="₹#,##0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -892,10 +892,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="2" t="n">
         <v>46239</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>50</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -905,10 +905,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="2" t="n">
         <v>46239</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -934,7 +934,7 @@
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1095,11 +1095,13 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:150.0, AS:150.0, AD:150.0</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
+          <t>C:0.0, AS:0.0, AD:0.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mismatch</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1406,202 +1408,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="5" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Node Name</t>
+          <t>camp_norm</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ad Account</t>
+          <t>Spend</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Spend</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>CPL</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>CPL</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Conversion Rate %</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Rate %</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Profit</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Profit</t>
+          <t>ROAS</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ROAS</t>
+          <t>ROI %</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>ROI %</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>CAC</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>Profitable?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ads</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ads2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1611,466 +1493,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="5" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Node Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ad Account</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Spend</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Leads</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>CPL</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Conversion Rate %</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ROAS</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>ROI %</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>CAC</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Profitable?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ads &gt; </t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ads2 &gt; </t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="5" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Node Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ad Account</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Spend</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Leads</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>CPL</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Conversion Rate %</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ROAS</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>ROI %</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>CAC</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Profitable?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ads &gt;  &gt; </t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ads2 &gt;  &gt; </t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2097,12 +1519,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Node Name</t>
+          <t>camp_norm</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ad Account</t>
+          <t>adset_norm</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2160,6 +1582,168 @@
           <t>Profitable?</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>camp_norm</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>adset_norm</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ad_norm</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CPL</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Conversion Rate %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ROI %</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Profitable?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: add all remaining source files, scripts, and documentation
</commit_message>
<xml_diff>
--- a/dummy.xlsx
+++ b/dummy.xlsx
@@ -29,8 +29,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="₹#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -866,12 +866,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -890,12 +891,17 @@
           <t>campaign</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source_file_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>46239</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>50</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -903,18 +909,24 @@
           <t>ads</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>46239</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>ads2</t>
         </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -934,7 +946,7 @@
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1087,7 +1099,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1095,13 +1107,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:0.0, AS:0.0, AD:0.0</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Mismatch</t>
-        </is>
+          <t>C:150.0, AS:0.0, AD:0.0</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1408,82 +1418,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>camp_norm</t>
+          <t>Node Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Ad Account</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CPL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Conversion Rate %</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ROAS</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ROI %</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>CAC</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Profitable?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ads</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ads2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1736,14 +1866,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Node Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ad Account</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CPL</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Conversion Rate %</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ROI %</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Profitable?</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix verification assertion for empty pipeline tests and final golden metrics implementation
</commit_message>
<xml_diff>
--- a/dummy.xlsx
+++ b/dummy.xlsx
@@ -940,12 +940,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -1330,6 +1330,422 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Count of sales that still lack a valid sale date</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>G. Total Sales</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>52</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>52</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Total Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>G. Attributed Sales</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>49</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>49</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Attributed Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>G. Unattributed Sales</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Unattributed Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>G. Total Revenue</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>467948</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>467948</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Total Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>G. Attributed Revenue</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>440951</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>440951</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Attributed Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>G. Unattributed Revenue</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>26997</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>26997</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Unattributed Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>G. Raw Meta Spend</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>456047.55</v>
+      </c>
+      <c r="D21" t="n">
+        <v>150</v>
+      </c>
+      <c r="E21" t="n">
+        <v>455897.55</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Raw Meta Spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>G. Attributed Spend</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>282120.59</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>282120.59</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Attributed Spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>G. Unallocated Spend</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>173926.96</v>
+      </c>
+      <c r="D23" t="n">
+        <v>150</v>
+      </c>
+      <c r="E23" t="n">
+        <v>173776.96</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Unallocated Spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>G. Profit</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>158830.41</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>158830.41</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Golden Report verification for Profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>G. ROAS</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Golden Report verification for ROAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>G. ROI %</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Golden Report verification for ROI %</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>G. CAC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>5757.56</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5757.56</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Golden Report verification for CAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>INV. Revenue Formula</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Attributed + Unattributed = Total Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>INV. Spend Formula</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Attributed + Unallocated = Raw Spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>INV. Profit Formula</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Attributed Revenue - Attributed Spend = Profit</t>
         </is>
       </c>
     </row>
@@ -1826,14 +2242,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Raw Meta Spend</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Attributed Spend</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unallocated Spend</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>150</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1846,14 +2302,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Funnel Stage</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Leads</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Paid Leads</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unpaid Leads</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1866,7 +2362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1951,6 +2447,120 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ads</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ads2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>